<commit_message>
feat: guruh rahbari va qabul eksportlariga so'rovnoma manzili, qatnov holati va guruh ustunlarini kiritish
</commit_message>
<xml_diff>
--- a/hisobotlar/qabul/QABUL - 2026.xlsx
+++ b/hisobotlar/qabul/QABUL - 2026.xlsx
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>996810119</v>
+        <v>884808270</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>978550581</v>
@@ -561,7 +561,11 @@
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Qaynar MFY, Mingbuloq koʻchasi, 90-uy</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 28-sonli umumiy o'rta ta'lim maktabi</t>
@@ -613,17 +617,21 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>885888187</v>
+        <v>24337740</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>902433774</v>
+        <v>858881870</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Guliston MFY, Buyuk ipak yoʻli, 115-uy</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 4-sonli umumiy o'rta ta'lim maktabi</t>
@@ -675,15 +683,21 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>953672602</v>
-      </c>
-      <c r="G6" s="2" t="n"/>
+        <v>536726020</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>906161560</v>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Ipak yuli MFY, Ipak yuli kuchasi, 12-uy</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 15-sonli umumiy o'rta ta'lim maktabi</t>
@@ -734,14 +748,22 @@
           <t>AE1520971</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
+      <c r="F7" s="2" t="n">
+        <v>701202208</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>701252208</v>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Xazara MFY, Hurriyat koʻchasi, 50-uy</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 39-sonli umumiy o'rta ta'lim maktabi</t>
@@ -793,15 +815,21 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>914606562</v>
-      </c>
-      <c r="G8" s="2" t="n"/>
+        <v>121770090</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>65620200</v>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Namaton MFY, Qoʻshchinor, 165 - uy</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 26-sonli umumiy o'rta ta'lim maktabi</t>
@@ -853,15 +881,21 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
+        <v>749526080</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>973873803</v>
       </c>
-      <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz shahri</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Dõstlik MFY, Bunyodkor kõchasi, 66/16-uy</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 14-sonli umumiy o'rta ta'lim maktabi</t>
@@ -913,15 +947,21 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>943387727</v>
-      </c>
-      <c r="G10" s="2" t="n"/>
+        <v>918108191</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>900995763</v>
+      </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Sevaz MFY, Kuxna bug'ot kuchasi, 73-uy</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Kitob qishloq xo'jalik kasb-hunar kolleji</t>
@@ -972,14 +1012,22 @@
           <t>AB9495274</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
+      <c r="F11" s="2" t="n">
+        <v>838893260</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>968513210</v>
+      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Boğishamol mahallasi, Uzbekistan kuchasi, 77 uy</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz Tibbiyot Kolleji</t>
@@ -1031,17 +1079,21 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
+        <v>775119810</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>919490180</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>877511981</v>
-      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Turon MFY, Turon koʻchasi, 17-uy</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 14-sonli umumiy o'rta ta'lim maktabi</t>
@@ -1093,17 +1145,21 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>509071311</v>
+        <v>90713110</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>500331311</v>
+        <v>973808965</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Maʼrifat MFY, Alpomish koʻchasi, 115-uy</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 7-sonli umumiy o'rta ta'lim maktabi</t>
@@ -1155,15 +1211,21 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>908788108</v>
-      </c>
-      <c r="G14" s="2" t="n"/>
+        <v>6673090</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>703902308</v>
+      </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Boston MFY, Abdulla Qodiriy köchasi, 31-uy</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 1-sonli umumiy o'rta ta'lim maktabi</t>
@@ -1215,17 +1277,21 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
+        <v>756108880</v>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>936031585</v>
       </c>
-      <c r="G15" s="2" t="n">
-        <v>882651585</v>
-      </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Duxchi MFY, Duxchi qishlog'i, 148.0</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 2-sonli umumiy o'rta ta'lim maktabi</t>
@@ -1277,17 +1343,21 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>910707501</v>
+        <v>107075010</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>908698209</v>
+        <v>86982090</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz shahri</t>
         </is>
       </c>
-      <c r="I16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Dòstlik MFY, Dòstlik kuchasi, 19-uy</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 2-son politexnikumi</t>
@@ -1339,15 +1409,21 @@
         </is>
       </c>
       <c r="F17" s="2" t="n">
+        <v>122400180</v>
+      </c>
+      <c r="G17" s="2" t="n">
         <v>912240018</v>
       </c>
-      <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Sinabog' M F Y, Sinabog' mahallasi, 101-uy</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 14-sonli umumiy o'rta ta'lim maktabi</t>
@@ -1399,15 +1475,21 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>700343131</v>
-      </c>
-      <c r="G18" s="2" t="n"/>
+        <v>3431310</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>3431310</v>
+      </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Qarshi tumani</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="n"/>
+          <t>Qashqadaryo, Kitob tumani</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Guluston, Guluston, 4.0</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
           <t>Qarshi pedagogika kolleji</t>
@@ -1459,15 +1541,21 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>770629890</v>
-      </c>
-      <c r="G19" s="2" t="n"/>
+        <v>706298900</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>973196260</v>
+      </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Kesh MFY, Kalakon kucha, 91-uy</t>
+        </is>
+      </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz texnologiya kasb-hunar kolleji</t>
@@ -1519,17 +1607,19 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>886177860</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>914577860</v>
-      </c>
+        <v>976190215</v>
+      </c>
+      <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="n"/>
+          <t>Qashqadaryo, Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Pakkandi MFY, Safarabot, 29_uy</t>
+        </is>
+      </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 6-sonli umumiy o'rta ta'lim maktabi</t>
@@ -1588,10 +1678,14 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Kesh MFY, Kesh ko'chasi, 102-uy</t>
+        </is>
+      </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 7-sonli umumiy o'rta ta'lim maktabi</t>
@@ -1643,15 +1737,21 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>870102621</v>
-      </c>
-      <c r="G22" s="2" t="n"/>
+        <v>701026210</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>977011783</v>
+      </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I22" s="2" t="n"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Qurilish, Varganza shaharchasi, 220-uy</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 52-sonli umumiy o'rta ta'lim maktabi</t>
@@ -1703,15 +1803,21 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>875681508</v>
-      </c>
-      <c r="G23" s="2" t="n"/>
+        <v>756815080</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>885857068</v>
+      </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I23" s="2" t="n"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Yangizamon, Durmon koʻchasi, 136-uy</t>
+        </is>
+      </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 24-sonli umumiy o'rta ta'lim maktabi</t>
@@ -1825,17 +1931,21 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>881151031</v>
+        <v>811510310</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>881840585</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Zargarlik MFY, Yakdillik ko'chasi, 186-uy</t>
+        </is>
+      </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 15-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2009,15 +2119,21 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>880880124</v>
-      </c>
-      <c r="G28" s="2" t="n"/>
+        <v>808801240</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>156130020</v>
+      </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I28" s="2" t="n"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Sevaz MFY, Taraqqiyot kuchasi, 130-uy</t>
+        </is>
+      </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 45-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2068,14 +2184,22 @@
           <t>AE5088010</t>
         </is>
       </c>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
+      <c r="F29" s="2" t="n">
+        <v>184403080</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>195942150</v>
+      </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Chiroqchi tumani</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="n"/>
+          <t>Qashqadaryo, Qiziltepa tumani</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Yuksalish mfy, Roxat koʻchasi, 44.0</t>
+        </is>
+      </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
           <t>Chiroqchi tumani 70-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2126,14 +2250,22 @@
           <t>AB7137876</t>
         </is>
       </c>
-      <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
+      <c r="F30" s="2" t="n">
+        <v>721302400</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>861885800</v>
+      </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I30" s="2" t="n"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Palandara MFY, Oftobroʻya qishlogʻi, 35.0</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Kitob agrobiznes kasb-hunar kolleji</t>
@@ -2185,17 +2317,21 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>975855793</v>
+        <v>776070824</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>776070824</v>
+        <v>739901790</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Ipak Yuli, Ipak Yuli, 118/26</t>
+        </is>
+      </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 15-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2305,17 +2441,21 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
+        <v>701080829</v>
+      </c>
+      <c r="G33" s="2" t="n">
         <v>992460829</v>
       </c>
-      <c r="G33" s="2" t="n">
-        <v>701080829</v>
-      </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Abziyat MFY, Bahor kuchasi, 62_-uy</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 34-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2427,17 +2567,21 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>908785105</v>
+        <v>87851050</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>916397685</v>
+        <v>163976850</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="n"/>
+          <t>Qashqadaryo, Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Taraģay, Chuyut, 153-uy</t>
+        </is>
+      </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri ixtisoslashtirilgan maktabi</t>
@@ -2488,14 +2632,22 @@
           <t>AE5324961</t>
         </is>
       </c>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
+      <c r="F36" s="2" t="n">
+        <v>505054080</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>906262080</v>
+      </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Chiroqchi tumani</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="n"/>
+          <t>Qashqadaryo, Qamashi tumani</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Yuksalish MFY, Olmazor, 183.0</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
           <t>Chiroqchi tumani 70-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2547,17 +2699,21 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>976312909</v>
+        <v>163545560</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>953332960</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Turon, Zarafshon, 12.01</t>
+        </is>
+      </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 26-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2669,17 +2825,21 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
+        <v>704897375</v>
+      </c>
+      <c r="G39" s="2" t="n">
         <v>770578758</v>
       </c>
-      <c r="G39" s="2" t="n">
-        <v>704897375</v>
-      </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Shanbe MFY, Chorvodor koʻcha, 10 uy</t>
+        </is>
+      </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 29-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2789,15 +2949,21 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>200132207</v>
-      </c>
-      <c r="G41" s="2" t="n"/>
+        <v>770850627</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>880850627</v>
+      </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Ipak yo’li, Ipak yo’li, 118/28</t>
+        </is>
+      </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 6-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2849,15 +3015,21 @@
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>996152272</v>
-      </c>
-      <c r="G42" s="2" t="n"/>
+        <v>794119200</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>961522720</v>
+      </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I42" s="2" t="n"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Zarafshon MFY, Yangiobod shaharchasi, 432.0</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani agrobiznes va xizmat ko'rsatish kasb-hunar kolleji</t>
@@ -2909,17 +3081,21 @@
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>885890027</v>
+        <v>886899080</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>957701169</v>
+        <v>577011690</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Shanbe MFY, Shabboda, 35 -uy</t>
+        </is>
+      </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 29-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2971,15 +3147,21 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>880115819</v>
-      </c>
-      <c r="G44" s="2" t="n"/>
+        <v>801158190</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>505870874</v>
+      </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I44" s="2" t="n"/>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Boģbon MFY, Ochamayli kòchasi, 100-uy</t>
+        </is>
+      </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 11-sonli umumiy o'rta ta'lim maktabi</t>
@@ -3031,17 +3213,21 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>916499228</v>
+        <v>146492280</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>976015200</v>
+        <v>886015200</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Qarshi tumani</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Kesh MFY, Do'stlik ko'chasi, 31/9-dom</t>
+        </is>
+      </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
           <t>Qarshi iqtisodiyot kolleji</t>
@@ -3093,15 +3279,21 @@
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>995658681</v>
-      </c>
-      <c r="G46" s="2" t="n"/>
+        <v>593907050</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>991437903</v>
+      </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I46" s="2" t="n"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Navbaxor MFY, Bolton qaychili, 99-uy</t>
+        </is>
+      </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 70-sonli umumiy o'rta ta'lim maktabi</t>
@@ -3153,17 +3345,21 @@
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>880669272</v>
+        <v>736908720</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>952556670</v>
+        <v>806692720</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>Shanbe MFY, Chorvador ko'chasi, 36-uy</t>
+        </is>
+      </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 29-sonli umumiy o'rta ta'lim maktabi</t>
@@ -3218,14 +3414,18 @@
         <v>334948423</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>991840519</v>
+        <v>494842333</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>G'arov, G'arov kuchasi, 84.0</t>
+        </is>
+      </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 19-sonli umumiy o'rta ta'lim maktabi</t>
@@ -3277,17 +3477,21 @@
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>700720614</v>
+        <v>7206140</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>992558990</v>
+        <v>577415640</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I49" s="2" t="n"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>Jilisuv QFY, Chimboy, 19 uy</t>
+        </is>
+      </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
           <t>Kitob agroservis xizmat ko'rsatish kasb-hunar kolleji</t>
@@ -3339,15 +3543,21 @@
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>880088028</v>
-      </c>
-      <c r="G50" s="2" t="n"/>
+        <v>700880280</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>880280880</v>
+      </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="n"/>
+          <t>Qashqadaryo, Kitob tumani</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Bo'ston mahallaa, Shodlik kuchasi, 140 uy</t>
+        </is>
+      </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 29-sonli umumiy o'rta ta'lim maktabi</t>
@@ -3519,15 +3729,21 @@
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>940790106</v>
-      </c>
-      <c r="G53" s="2" t="n"/>
+        <v>407901060</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>351375740</v>
+      </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="n"/>
+          <t>Qashqadaryo, Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Galabek MFY, Maftunkor koʻchasi, 39-uy</t>
+        </is>
+      </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 50-sonli umumiy o'rta ta'lim maktabi</t>
@@ -3639,15 +3855,21 @@
         </is>
       </c>
       <c r="F55" s="2" t="n">
+        <v>705180560</v>
+      </c>
+      <c r="G55" s="2" t="n">
         <v>997307709</v>
       </c>
-      <c r="G55" s="2" t="n"/>
       <c r="H55" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Yakkabog' tumani</t>
         </is>
       </c>
-      <c r="I55" s="2" t="n"/>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Kattabogʻ MFY, Mardona koʻchasi, 56-uy</t>
+        </is>
+      </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
           <t>Yakkabog' tumani 43-sonli umumiy o'rta ta'lim maktabi</t>
@@ -3823,17 +4045,21 @@
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>999430596</v>
+        <v>593992050</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>959399205</v>
+        <v>523327660</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I58" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Gelon MFY, Gelon, 43uy</t>
+        </is>
+      </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 58-sonli umumiy o'rta ta'lim maktabi</t>
@@ -3885,15 +4111,21 @@
         </is>
       </c>
       <c r="F59" s="2" t="n">
+        <v>45042400</v>
+      </c>
+      <c r="G59" s="2" t="n">
         <v>939034744</v>
       </c>
-      <c r="G59" s="2" t="n"/>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
-        </is>
-      </c>
-      <c r="I59" s="2" t="n"/>
+          <t>Qashqadaryo viloyati</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Alaquyliq MFY, Mevali koʻchasi, 85-uy</t>
+        </is>
+      </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 20-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4123,17 +4355,21 @@
         </is>
       </c>
       <c r="F63" s="2" t="n">
+        <v>780066370</v>
+      </c>
+      <c r="G63" s="2" t="n">
         <v>970012780</v>
       </c>
-      <c r="G63" s="2" t="n">
-        <v>973157721</v>
-      </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I63" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Yangibogʻ MFY, Mirzo Ulugʻbek koʼchasi, 41-uy</t>
+        </is>
+      </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 19-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4188,14 +4424,18 @@
         <v>772131924</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>919584082</v>
+        <v>548408291</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Hisorak MFY, Duoba qishlog'i, 1 - uy</t>
+        </is>
+      </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 61-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4254,10 +4494,14 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Oq Oltin MFY, Al-Xorazmiy koʼchasi, 212-uy</t>
+        </is>
+      </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 68-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4371,7 +4615,7 @@
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>503019503</v>
+        <v>501582729</v>
       </c>
       <c r="G67" s="2" t="n">
         <v>997304804</v>
@@ -4381,7 +4625,11 @@
           <t>Qashqadaryo, Shahrisabz shahri</t>
         </is>
       </c>
-      <c r="I67" s="2" t="n"/>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Turon MFY, Turon koʻchasi, 52.0</t>
+        </is>
+      </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 49-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4433,15 +4681,21 @@
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>919595774</v>
-      </c>
-      <c r="G68" s="2" t="n"/>
+        <v>195957710</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>919595771</v>
+      </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I68" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Oq oltin MFY, Mehnatsevar kòchasi, 39-uy</t>
+        </is>
+      </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 68-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4493,7 +4747,7 @@
         </is>
       </c>
       <c r="F69" s="2" t="n">
-        <v>880632608</v>
+        <v>806326080</v>
       </c>
       <c r="G69" s="2" t="n">
         <v>973360140</v>
@@ -4503,7 +4757,11 @@
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I69" s="2" t="n"/>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Charmgar MFY, Nomozgoh ko'chasi, 124-uy</t>
+        </is>
+      </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 4-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4675,17 +4933,21 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>330578323</v>
+        <v>47809270</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>334248323</v>
+        <v>305783230</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I72" s="2" t="n"/>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>Obod MFY, Qushboshi, 6-uy</t>
+        </is>
+      </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 38-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4737,7 +4999,7 @@
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>885020703</v>
+        <v>850207030</v>
       </c>
       <c r="G73" s="2" t="n">
         <v>880037679</v>
@@ -4747,7 +5009,11 @@
           <t>Qashqadaryo, Yakkabog' tumani</t>
         </is>
       </c>
-      <c r="I73" s="2" t="n"/>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>Chagʼatoy, Yuq, 76.0</t>
+        </is>
+      </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
           <t>Yakkabog' tumani 69-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4801,13 +5067,19 @@
       <c r="F74" s="2" t="n">
         <v>704785808</v>
       </c>
-      <c r="G74" s="2" t="n"/>
+      <c r="G74" s="2" t="n">
+        <v>887538486</v>
+      </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>Sanam MFY, Uzumzor kochasi, 60.0</t>
+        </is>
+      </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 1-son texnikumi</t>
@@ -4859,15 +5131,21 @@
         </is>
       </c>
       <c r="F75" s="2" t="n">
-        <v>955838858</v>
-      </c>
-      <c r="G75" s="2" t="n"/>
+        <v>558388580</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>916417532</v>
+      </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I75" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>Hisorak MFY, Chungurak qishloği, 132-uy</t>
+        </is>
+      </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 61-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4919,17 +5197,21 @@
         </is>
       </c>
       <c r="F76" s="2" t="n">
+        <v>874853608</v>
+      </c>
+      <c r="G76" s="2" t="n">
         <v>971880757</v>
       </c>
-      <c r="G76" s="2" t="n">
-        <v>973810757</v>
-      </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I76" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>Bog'ishamol MFY, Sa‘d Ibn vaqqos ko‘chasi, 33 -uy</t>
+        </is>
+      </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 26-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4981,15 +5263,21 @@
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>887611310</v>
-      </c>
-      <c r="G77" s="2" t="n"/>
+        <v>876113100</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>738982040</v>
+      </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I77" s="2" t="n"/>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>Рус кишлак МФЮ, Улица Рус кишлак, Дом-11</t>
+        </is>
+      </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 25-sonli umumiy o'rta ta'lim maktabi</t>
@@ -5110,10 +5398,14 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
-        </is>
-      </c>
-      <c r="I79" s="2" t="n"/>
+          <t>Qashqadaryo, Китоб</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>китоб МФЯ, гулустон кучаси, 90.0</t>
+        </is>
+      </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 12-sonli umumiy o'rta ta'lim maktabi</t>
@@ -5165,17 +5457,21 @@
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>888659008</v>
+        <v>898183800</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>881861712</v>
+        <v>883861712</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I80" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>Bogʻishamol MFY, Qorapoycha, 6 uy</t>
+        </is>
+      </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 26-sonli umumiy o'rta ta'lim maktabi</t>
@@ -5227,15 +5523,21 @@
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>772254208</v>
-      </c>
-      <c r="G81" s="2" t="n"/>
+        <v>722542080</v>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>994513820</v>
+      </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I81" s="2" t="n"/>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>Sanam MFY, Shahrisabz koʻchasi, 163-uy</t>
+        </is>
+      </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 1-son texnikumi</t>
@@ -5287,17 +5589,21 @@
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>908785105</v>
+        <v>862338080</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>916397685</v>
+        <v>770216705</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
-        </is>
-      </c>
-      <c r="I82" s="2" t="n"/>
+          <t>Qashqadaryo, Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Qirgʻiz MFY, Ming terak koʻchasi, 20-uy</t>
+        </is>
+      </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 36-sonli umumiy o'rta ta'lim maktabi</t>
@@ -5349,15 +5655,21 @@
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>997422473</v>
-      </c>
-      <c r="G83" s="2" t="n"/>
+        <v>514708250</v>
+      </c>
+      <c r="G83" s="2" t="n">
+        <v>224730951</v>
+      </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Yakkabog' tumani</t>
         </is>
       </c>
-      <c r="I83" s="2" t="n"/>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>Kenguzar MFY, Chig'atoy, 6.0</t>
+        </is>
+      </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
           <t>Yakkabog' tumani 69-sonli umumiy o'rta ta'lim maktabi</t>
@@ -5409,17 +5721,21 @@
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>881708081</v>
+        <v>804102270</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>880410227</v>
+        <v>817080810</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I84" s="2" t="n"/>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Xoji MFY, Uzunqir kuchasi, 106.0</t>
+        </is>
+      </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 12-sonli umumiy o'rta ta'lim maktabi</t>
@@ -5533,17 +5849,21 @@
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>991312508</v>
+        <v>913125080</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>880068282</v>
+        <v>760782870</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I86" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>Kichik novqat mfy, Soyboʻyi koʻchasi, 04</t>
+        </is>
+      </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 9-sonli umumiy o'rta ta'lim maktabi</t>
@@ -5595,15 +5915,21 @@
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>930190686</v>
-      </c>
-      <c r="G87" s="2" t="n"/>
+        <v>33187080</v>
+      </c>
+      <c r="G87" s="2" t="n">
+        <v>11906860</v>
+      </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
-        </is>
-      </c>
-      <c r="I87" s="2" t="n"/>
+          <t>Qashqadaryo, Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>Quruq soy MFY, Buzovut qishlogʻi, 111-uy</t>
+        </is>
+      </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 96-sonli umumiy o'rta ta'lim maktabi</t>
@@ -5717,17 +6043,21 @@
         </is>
       </c>
       <c r="F89" s="2" t="n">
-        <v>875910918</v>
+        <v>759109180</v>
       </c>
       <c r="G89" s="2" t="n">
         <v>885660802</v>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I89" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>Uymovut MFY, Qadriyat ko'chasi, 127-uy</t>
+        </is>
+      </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 2-sonli umumiy o'rta ta'lim maktabi</t>
@@ -5779,15 +6109,21 @@
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>906752661</v>
-      </c>
-      <c r="G90" s="2" t="n"/>
+        <v>763104770</v>
+      </c>
+      <c r="G90" s="2" t="n">
+        <v>732104770</v>
+      </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I90" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>Bunyodkor, Sadriddin ayni, 6_uy</t>
+        </is>
+      </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 14-sonli umumiy o'rta ta'lim maktabi</t>
@@ -5842,14 +6178,18 @@
         <v>991863023</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>952282462</v>
+        <v>991863023</v>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I91" s="2" t="n"/>
+          <t>Qashqadaryo, Yakkabog' tumani</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>Alakuylak MFY, Hamid Olimjon koʻchasi, 55.0</t>
+        </is>
+      </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz pedagogika va turizm kasb-hunar kolleji</t>
@@ -5973,7 +6313,11 @@
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I93" s="2" t="n"/>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>Hamid Olimjon, Hamid Olimjon 213, 213uy</t>
+        </is>
+      </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 1-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6087,15 +6431,21 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>995264709</v>
-      </c>
-      <c r="G95" s="2" t="n"/>
+        <v>834030080</v>
+      </c>
+      <c r="G95" s="2" t="n">
+        <v>952647090</v>
+      </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
-        </is>
-      </c>
-      <c r="I95" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>Guliston MFY, Qoʻshtepa kòchasi, 329.0</t>
+        </is>
+      </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 5-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6146,14 +6496,22 @@
           <t>AE4994200</t>
         </is>
       </c>
-      <c r="F96" s="2" t="n"/>
-      <c r="G96" s="2" t="n"/>
+      <c r="F96" s="2" t="n">
+        <v>1114090</v>
+      </c>
+      <c r="G96" s="2" t="n">
+        <v>973891174</v>
+      </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I96" s="2" t="n"/>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>Charimgar MFY, Navoiy kucha, 44uy</t>
+        </is>
+      </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 4-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6205,17 +6563,21 @@
         </is>
       </c>
       <c r="F97" s="2" t="n">
-        <v>904403666</v>
+        <v>44036660</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>912204218</v>
+        <v>122477210</v>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I97" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>Fayzobod MFY, Yangi kesh, 242-uy</t>
+        </is>
+      </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz yengil sanoat va xizmat ko'rsatish kasb-hunar kolleji</t>
@@ -6267,17 +6629,21 @@
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>880306601</v>
+        <v>884943800</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>970874905</v>
+        <v>880449802</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I98" s="2" t="n"/>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>Iskana MFY, Uchtepalik, 52.0</t>
+        </is>
+      </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 51-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6329,15 +6695,21 @@
         </is>
       </c>
       <c r="F99" s="2" t="n">
-        <v>505899948</v>
-      </c>
-      <c r="G99" s="2" t="n"/>
+        <v>58999480</v>
+      </c>
+      <c r="G99" s="2" t="n">
+        <v>73473860</v>
+      </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I99" s="2" t="n"/>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>Sho'robsoy MFY, Komillik ko'chasi, 18uy</t>
+        </is>
+      </c>
       <c r="J99" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 23-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6389,15 +6761,21 @@
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>900709579</v>
-      </c>
-      <c r="G100" s="2" t="n"/>
+        <v>874637908</v>
+      </c>
+      <c r="G100" s="2" t="n">
+        <v>107095790</v>
+      </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I100" s="2" t="n"/>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>Beshqazoq MFY, Oq daryo, 56-uy</t>
+        </is>
+      </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 6-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6449,17 +6827,21 @@
         </is>
       </c>
       <c r="F101" s="2" t="n">
-        <v>991682082</v>
+        <v>916820820</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>770427406</v>
+        <v>916820820</v>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Yakkabog' tumani</t>
         </is>
       </c>
-      <c r="I101" s="2" t="n"/>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>Qoʻshchinor, AbulqosimFirdavsiy, 22-uy</t>
+        </is>
+      </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
           <t>Yakkabog' tumani 70-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6511,15 +6893,21 @@
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>908841208</v>
-      </c>
-      <c r="G102" s="2" t="n"/>
+        <v>88412080</v>
+      </c>
+      <c r="G102" s="2" t="n">
+        <v>195727170</v>
+      </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I102" s="2" t="n"/>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>Uluğbek MFY, Mirzo Tursunzoda kòchasi, 49.0</t>
+        </is>
+      </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 32-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6571,17 +6959,21 @@
         </is>
       </c>
       <c r="F103" s="2" t="n">
-        <v>888270718</v>
+        <v>883879404</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>883860485</v>
+        <v>883813979</v>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I103" s="2" t="n"/>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>Yakatut MFY, Kumirtepa kuchasi, 60uy</t>
+        </is>
+      </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 18-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6691,15 +7083,21 @@
         </is>
       </c>
       <c r="F105" s="2" t="n">
-        <v>908780280</v>
-      </c>
-      <c r="G105" s="2" t="n"/>
+        <v>87802800</v>
+      </c>
+      <c r="G105" s="2" t="n">
+        <v>526948780</v>
+      </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I105" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>Xitoy MFY, Besh chinor, 65.0</t>
+        </is>
+      </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 56-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6751,17 +7149,21 @@
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>883367774</v>
+        <v>833677740</v>
       </c>
       <c r="G106" s="2" t="n">
         <v>907163142</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I106" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>Do'stlik MFY, Bunyodkor ko'chasi, 62/16-uy</t>
+        </is>
+      </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 14-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6873,15 +7275,21 @@
         </is>
       </c>
       <c r="F108" s="2" t="n">
+        <v>702902740</v>
+      </c>
+      <c r="G108" s="2" t="n">
         <v>882633833</v>
       </c>
-      <c r="G108" s="2" t="n"/>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I108" s="2" t="n"/>
+          <t>Qashqadaryo, Kitob tumani</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>Guliston MFY, Qo'shtepa mahallasi, 75.0</t>
+        </is>
+      </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 5-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6933,17 +7341,21 @@
         </is>
       </c>
       <c r="F109" s="2" t="n">
-        <v>885872701</v>
+        <v>858727010</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>910704107</v>
+        <v>68720885</v>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I109" s="2" t="n"/>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>Hoʻjailimkoni MFY, Hoʻjailimkoni qishlogʻi, 248-uy</t>
+        </is>
+      </c>
       <c r="J109" s="2" t="inlineStr">
         <is>
           <t>Kitob qishloq xo'jalik kasb-hunar kolleji</t>
@@ -6995,15 +7407,21 @@
         </is>
       </c>
       <c r="F110" s="2" t="n">
-        <v>871160303</v>
-      </c>
-      <c r="G110" s="2" t="n"/>
+        <v>711603030</v>
+      </c>
+      <c r="G110" s="2" t="n">
+        <v>711603030</v>
+      </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I110" s="2" t="n"/>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>Homid Olimjom MFY, Amir Temur kochasi, 47 uy</t>
+        </is>
+      </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 1-sonli ayrim fanlar chuqur o'rganiladigan ixtisoslashtirilgan maktabi</t>
@@ -7065,7 +7483,11 @@
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I111" s="2" t="n"/>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>Obikanda MFY, Baland Tepa koʻchasi, 23-uy</t>
+        </is>
+      </c>
       <c r="J111" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 63-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7117,15 +7539,21 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>879340301</v>
-      </c>
-      <c r="G112" s="2" t="n"/>
+        <v>793403010</v>
+      </c>
+      <c r="G112" s="2" t="n">
+        <v>872288840</v>
+      </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I112" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>Xonabod MFY, Samarqand kuchasi, 85-uy</t>
+        </is>
+      </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 60-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7301,17 +7729,21 @@
         </is>
       </c>
       <c r="F115" s="2" t="n">
-        <v>701202277</v>
+        <v>68161770</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>880096166</v>
+        <v>961660883</v>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I115" s="2" t="n"/>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>Xalqlar do'stligi MFY, Qashqadaryo2, 65.0</t>
+        </is>
+      </c>
       <c r="J115" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 3-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7425,17 +7857,21 @@
         </is>
       </c>
       <c r="F117" s="2" t="n">
-        <v>908785105</v>
+        <v>311580830</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>916397685</v>
+        <v>883800339</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I117" s="2" t="n"/>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>Bogʻibaland MFY, Xirmanjoy kòchasi, 121-uy</t>
+        </is>
+      </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 53-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7547,7 +7983,7 @@
         </is>
       </c>
       <c r="F119" s="2" t="n">
-        <v>333890503</v>
+        <v>338905030</v>
       </c>
       <c r="G119" s="2" t="n">
         <v>949791283</v>
@@ -7557,7 +7993,11 @@
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I119" s="2" t="n"/>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>Oq suv MFY, Nimgi koʻchasi, 69-uy</t>
+        </is>
+      </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 46-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7671,17 +8111,21 @@
         </is>
       </c>
       <c r="F121" s="2" t="n">
-        <v>774231707</v>
+        <v>743217070</v>
       </c>
       <c r="G121" s="2" t="n">
-        <v>956162509</v>
+        <v>561635090</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
-        </is>
-      </c>
-      <c r="I121" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>Bektemir MFY, Shifokorlar kuchasi, 238-uy</t>
+        </is>
+      </c>
       <c r="J121" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 21-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7733,17 +8177,21 @@
         </is>
       </c>
       <c r="F122" s="2" t="n">
-        <v>883090228</v>
+        <v>830902280</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>886177808</v>
+        <v>800578080</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz shahri</t>
         </is>
       </c>
-      <c r="I122" s="2" t="n"/>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>G'alaba MFY, Firdavsiy ko'chasi, 12/2-uy</t>
+        </is>
+      </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 2-son politexnikumi</t>
@@ -7795,15 +8243,21 @@
         </is>
       </c>
       <c r="F123" s="2" t="n">
-        <v>914551195</v>
-      </c>
-      <c r="G123" s="2" t="n"/>
+        <v>840204080</v>
+      </c>
+      <c r="G123" s="2" t="n">
+        <v>990630419</v>
+      </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I123" s="2" t="n"/>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
+          <t>Navbahor MFY, Eski Jilisuv 3 qishlog‘i, 92-uy</t>
+        </is>
+      </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 2-son texnikumi</t>
@@ -7917,17 +8371,21 @@
         </is>
       </c>
       <c r="F125" s="2" t="n">
-        <v>887381981</v>
+        <v>762945080</v>
       </c>
       <c r="G125" s="2" t="n">
-        <v>957401981</v>
+        <v>873819820</v>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I125" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>Toʻdamaydon, Fidokor, 92.0</t>
+        </is>
+      </c>
       <c r="J125" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 43-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7979,17 +8437,21 @@
         </is>
       </c>
       <c r="F126" s="2" t="n">
-        <v>886199703</v>
+        <v>818311670</v>
       </c>
       <c r="G126" s="2" t="n">
-        <v>876295108</v>
+        <v>183116787</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I126" s="2" t="n"/>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>Iskana MFY, Iskana ko'chasi, 40-uy</t>
+        </is>
+      </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 51-sonli umumiy o'rta ta'lim maktabi</t>
@@ -8041,15 +8503,21 @@
         </is>
       </c>
       <c r="F127" s="2" t="n">
-        <v>936367986</v>
-      </c>
-      <c r="G127" s="2" t="n"/>
+        <v>793476080</v>
+      </c>
+      <c r="G127" s="2" t="n">
+        <v>914564661</v>
+      </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I127" s="2" t="n"/>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
+          <t>BektimirMFY, Yoshlar kuchasi, 27.0</t>
+        </is>
+      </c>
       <c r="J127" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 21-sonli umumiy o'rta ta'lim maktabi</t>
@@ -8161,15 +8629,21 @@
         </is>
       </c>
       <c r="F129" s="2" t="n">
-        <v>978577404</v>
-      </c>
-      <c r="G129" s="2" t="n"/>
+        <v>978527404</v>
+      </c>
+      <c r="G129" s="2" t="n">
+        <v>785274040</v>
+      </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Qarshi tumani</t>
-        </is>
-      </c>
-      <c r="I129" s="2" t="n"/>
+          <t>Qashqadaryo, Kitob tumani</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>Katlos mfy, Obigarm kuchasi, 89.0</t>
+        </is>
+      </c>
       <c r="J129" s="2" t="inlineStr">
         <is>
           <t>Qarshi pedagogika kolleji</t>
@@ -8221,17 +8695,21 @@
         </is>
       </c>
       <c r="F130" s="2" t="n">
-        <v>946034407</v>
+        <v>460344070</v>
       </c>
       <c r="G130" s="2" t="n">
-        <v>912138081</v>
+        <v>30150780</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Yakkabog' tumani</t>
         </is>
       </c>
-      <c r="I130" s="2" t="n"/>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>Chumich MFY, Ayg'irkul ko'chasi, 42-uy</t>
+        </is>
+      </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
           <t>Yakkabog' tumani 75-sonli umumiy o'rta ta'lim maktabi</t>
@@ -8344,14 +8822,22 @@
           <t>AD7829399</t>
         </is>
       </c>
-      <c r="F132" s="2" t="n"/>
-      <c r="G132" s="2" t="n"/>
+      <c r="F132" s="2" t="n">
+        <v>940693027</v>
+      </c>
+      <c r="G132" s="2" t="n">
+        <v>940693027</v>
+      </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I132" s="2" t="n"/>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>Shurabsoy MFY, Boshchil qishlogʼi, 68-uy</t>
+        </is>
+      </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
           <t>Kitob agrosanoat kasb-hunar kolleji</t>
@@ -8403,15 +8889,21 @@
         </is>
       </c>
       <c r="F133" s="2" t="n">
-        <v>886030021</v>
-      </c>
-      <c r="G133" s="2" t="n"/>
+        <v>881796080</v>
+      </c>
+      <c r="G133" s="2" t="n">
+        <v>530860888</v>
+      </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
-        </is>
-      </c>
-      <c r="I133" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>Miraki mfy, Navoiy ko'chasi, 68.0</t>
+        </is>
+      </c>
       <c r="J133" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 8-sonli umumiy o'rta ta'lim maktabi</t>
@@ -8584,14 +9076,22 @@
           <t>AE7082532</t>
         </is>
       </c>
-      <c r="F136" s="2" t="n"/>
-      <c r="G136" s="2" t="n"/>
+      <c r="F136" s="2" t="n">
+        <v>107102830</v>
+      </c>
+      <c r="G136" s="2" t="n">
+        <v>107102830</v>
+      </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I136" s="2" t="n"/>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>Hamid Olimjon MFY, Amir Temur, 69.0</t>
+        </is>
+      </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 1-sonli umumiy o'rta ta'lim maktabi</t>
@@ -8643,17 +9143,21 @@
         </is>
       </c>
       <c r="F137" s="2" t="n">
-        <v>973889978</v>
+        <v>738899780</v>
       </c>
       <c r="G137" s="2" t="n">
-        <v>880407877</v>
+        <v>755860880</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I137" s="2" t="n"/>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>Alaquyliq MFY, Tutzoz kuchasi, 16-uy</t>
+        </is>
+      </c>
       <c r="J137" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 20-sonli umumiy o'rta ta'lim maktabi</t>
@@ -8825,17 +9329,21 @@
         </is>
       </c>
       <c r="F140" s="2" t="n">
-        <v>995240810</v>
+        <v>910608100</v>
       </c>
       <c r="G140" s="2" t="n">
-        <v>955248180</v>
+        <v>781800701</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I140" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>Sayyod MFY, Obod mahallasi, 13.0</t>
+        </is>
+      </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 66-sonli umumiy o'rta ta'lim maktabi</t>
@@ -8887,17 +9395,21 @@
         </is>
       </c>
       <c r="F141" s="2" t="n">
-        <v>773900314</v>
+        <v>796563080</v>
       </c>
       <c r="G141" s="2" t="n">
-        <v>779656308</v>
+        <v>713906770</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I141" s="2" t="n"/>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>Surum mahallasi, Sokin koʻchasi, 66.0</t>
+        </is>
+      </c>
       <c r="J141" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 85-sonli umumiy o'rta ta'lim maktabi</t>
@@ -8949,17 +9461,21 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
+        <v>180216700</v>
+      </c>
+      <c r="G142" s="2" t="n">
         <v>919614037</v>
       </c>
-      <c r="G142" s="2" t="n">
-        <v>918021670</v>
-      </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I142" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>Sinabog’ MFY, Shoxsaroy ko’chasi, 205-uy</t>
+        </is>
+      </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 1-sonli umumiy o'rta ta'lim maktabi</t>
@@ -9011,17 +9527,21 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>908942471</v>
+        <v>86424710</v>
       </c>
       <c r="G143" s="2" t="n">
-        <v>919496471</v>
+        <v>194964710</v>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz shahri</t>
         </is>
       </c>
-      <c r="I143" s="2" t="n"/>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>Dustlik mahallasi, Bunyodkor kuchasi, 97.0</t>
+        </is>
+      </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 14-sonli ayrim fanlar chuqur o'rganiladigan ixtisoslashtirilgan maktabi</t>
@@ -9073,17 +9593,21 @@
         </is>
       </c>
       <c r="F144" s="2" t="n">
-        <v>919600814</v>
+        <v>196008140</v>
       </c>
       <c r="G144" s="2" t="n">
         <v>912250767</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I144" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>Zingiron MFY, Zingiron ko'chasi, 46-uy</t>
+        </is>
+      </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 15-sonli umumiy o'rta ta'lim maktabi</t>
@@ -9135,15 +9659,21 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>995658681</v>
-      </c>
-      <c r="G145" s="2" t="n"/>
+        <v>780982300</v>
+      </c>
+      <c r="G145" s="2" t="n">
+        <v>956586810</v>
+      </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I145" s="2" t="n"/>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>Navbahor MFY, Yangi jilisuv qishlogʻi, 99 uy</t>
+        </is>
+      </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 70-sonli umumiy o'rta ta'lim maktabi</t>
@@ -9195,15 +9725,21 @@
         </is>
       </c>
       <c r="F146" s="2" t="n">
-        <v>995658681</v>
-      </c>
-      <c r="G146" s="2" t="n"/>
+        <v>780981300</v>
+      </c>
+      <c r="G146" s="2" t="n">
+        <v>956586810</v>
+      </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I146" s="2" t="n"/>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>Jilisuv MFY, Yangi Jilisuv, 99.0</t>
+        </is>
+      </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 70-sonli umumiy o'rta ta'lim maktabi</t>
@@ -9255,15 +9791,21 @@
         </is>
       </c>
       <c r="F147" s="2" t="n">
-        <v>870004608</v>
-      </c>
-      <c r="G147" s="2" t="n"/>
+        <v>700046080</v>
+      </c>
+      <c r="G147" s="2" t="n">
+        <v>771088048</v>
+      </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I147" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>Bogʻishamol MFY, Oʻzbekiston koʻchasi, 15-uy</t>
+        </is>
+      </c>
       <c r="J147" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 26-sonli umumiy o'rta ta'lim maktabi</t>
@@ -9317,13 +9859,19 @@
       <c r="F148" s="2" t="n">
         <v>995590930</v>
       </c>
-      <c r="G148" s="2" t="n"/>
+      <c r="G148" s="2" t="n">
+        <v>518201950</v>
+      </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Yakkabog' tumani</t>
         </is>
       </c>
-      <c r="I148" s="2" t="n"/>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>Yangiobod mahhalla, Ezgulik kuchasi, 17B</t>
+        </is>
+      </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
           <t>Yakkabog' maishiy xizmat kasb-hunar kolleji</t>
@@ -9375,15 +9923,21 @@
         </is>
       </c>
       <c r="F149" s="2" t="n">
-        <v>914551195</v>
-      </c>
-      <c r="G149" s="2" t="n"/>
+        <v>48913000</v>
+      </c>
+      <c r="G149" s="2" t="n">
+        <v>908708827</v>
+      </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
-        </is>
-      </c>
-      <c r="I149" s="2" t="n"/>
+          <t>Qashqadaryo, Kitob tumani</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>Yangi obod MFY, Yangi obod 11/5, 11/5</t>
+        </is>
+      </c>
       <c r="J149" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 2-son texnikumi</t>
@@ -9435,17 +9989,21 @@
         </is>
       </c>
       <c r="F150" s="2" t="n">
-        <v>903410676</v>
+        <v>189804950</v>
       </c>
       <c r="G150" s="2" t="n">
-        <v>918980495</v>
+        <v>88308650</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I150" s="2" t="n"/>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>Saray MFY, Yangiqishloq, 81-uy</t>
+        </is>
+      </c>
       <c r="J150" s="2" t="inlineStr">
         <is>
           <t>Kitob iqtisodiyot kolleji</t>
@@ -9497,17 +10055,21 @@
         </is>
       </c>
       <c r="F151" s="2" t="n">
-        <v>971100325</v>
+        <v>887100325</v>
       </c>
       <c r="G151" s="2" t="n">
-        <v>910710683</v>
+        <v>884710683</v>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
-        </is>
-      </c>
-      <c r="I151" s="2" t="n"/>
+          <t>Qashqadaryo, Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>Qirğiz MFY, Yoshlik kõchasi, 29-uy</t>
+        </is>
+      </c>
       <c r="J151" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 36-sonli umumiy o'rta ta'lim maktabi</t>
@@ -9561,13 +10123,19 @@
       <c r="F152" s="2" t="n">
         <v>977997671</v>
       </c>
-      <c r="G152" s="2" t="n"/>
+      <c r="G152" s="2" t="n">
+        <v>884037671</v>
+      </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz shahri</t>
         </is>
       </c>
-      <c r="I152" s="2" t="n"/>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>Kesh, Kalokon, 73 uy</t>
+        </is>
+      </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 2-son kasb-hunar maktabi</t>
@@ -9626,10 +10194,14 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I153" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>Hojimaydon MFY, Chambil koʻchasi, 14-uy</t>
+        </is>
+      </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 7-sonli umumiy o'rta ta'lim maktabi</t>
@@ -9681,15 +10253,21 @@
         </is>
       </c>
       <c r="F154" s="2" t="n">
-        <v>887886042</v>
-      </c>
-      <c r="G154" s="2" t="n"/>
+        <v>878860420</v>
+      </c>
+      <c r="G154" s="2" t="n">
+        <v>916383271</v>
+      </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I154" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>Fayzobod MFY, Quruvchilar kuchasi, 68 uy</t>
+        </is>
+      </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz Yengil sanoat kasb-hunar kolleji</t>
@@ -9741,15 +10319,21 @@
         </is>
       </c>
       <c r="F155" s="2" t="n">
-        <v>919490481</v>
-      </c>
-      <c r="G155" s="2" t="n"/>
+        <v>198815080</v>
+      </c>
+      <c r="G155" s="2" t="n">
+        <v>904810912</v>
+      </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Yakkabog' tumani</t>
         </is>
       </c>
-      <c r="I155" s="2" t="n"/>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
+          <t>Darxon MFY, Eshonguzar, 52-uy</t>
+        </is>
+      </c>
       <c r="J155" s="2" t="inlineStr">
         <is>
           <t>Yakkabog' tumani 4-sonli umumiy o'rta ta'lim maktabi</t>
@@ -9921,17 +10505,21 @@
         </is>
       </c>
       <c r="F158" s="2" t="n">
-        <v>950202813</v>
+        <v>502028130</v>
       </c>
       <c r="G158" s="2" t="n">
-        <v>950702813</v>
+        <v>727528130</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I158" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I158" s="2" t="inlineStr">
+        <is>
+          <t>SinaboĝMFY, Sinaboĝ kuchasi, 133-uy</t>
+        </is>
+      </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 23-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10045,17 +10633,21 @@
         </is>
       </c>
       <c r="F160" s="2" t="n">
-        <v>996739929</v>
+        <v>967399290</v>
       </c>
       <c r="G160" s="2" t="n">
-        <v>973194003</v>
+        <v>967399290</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I160" s="2" t="n"/>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>Katlos MFY, Oshqon kuchasi, 69-uy</t>
+        </is>
+      </c>
       <c r="J160" s="2" t="inlineStr">
         <is>
           <t>Kitob agrobiznes kasb-hunar kolleji</t>
@@ -10167,7 +10759,7 @@
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>332960708</v>
+        <v>329607080</v>
       </c>
       <c r="G162" s="2" t="n">
         <v>881360926</v>
@@ -10177,7 +10769,11 @@
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I162" s="2" t="n"/>
+      <c r="I162" s="2" t="inlineStr">
+        <is>
+          <t>Sariosiyo MFY, Chinorlik ko'chasi, 14.0</t>
+        </is>
+      </c>
       <c r="J162" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 81-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10229,17 +10825,21 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>887326111</v>
+        <v>873261110</v>
       </c>
       <c r="G163" s="2" t="n">
-        <v>906176883</v>
+        <v>768830906</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I163" s="2" t="n"/>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
+          <t>Ulugʻbek MFY, Qizil darvoza kuchasi, 116.0</t>
+        </is>
+      </c>
       <c r="J163" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 32-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10353,17 +10953,21 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>883887912</v>
+        <v>771601300</v>
       </c>
       <c r="G165" s="2" t="n">
-        <v>877160130</v>
+        <v>838879120</v>
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I165" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I165" s="2" t="inlineStr">
+        <is>
+          <t>Uymovut MFY, Ohangrabo ko'chasi, 97-uy</t>
+        </is>
+      </c>
       <c r="J165" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 20-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10475,15 +11079,21 @@
         </is>
       </c>
       <c r="F167" s="2" t="n">
-        <v>876590027</v>
-      </c>
-      <c r="G167" s="2" t="n"/>
+        <v>765900270</v>
+      </c>
+      <c r="G167" s="2" t="n">
+        <v>707908680</v>
+      </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I167" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I167" s="2" t="inlineStr">
+        <is>
+          <t>Bunyodkor MFY, Paxtakor koʻchasi, 44/a</t>
+        </is>
+      </c>
       <c r="J167" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 7-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10592,14 +11202,22 @@
           <t>AD9706738</t>
         </is>
       </c>
-      <c r="F169" s="2" t="n"/>
-      <c r="G169" s="2" t="n"/>
+      <c r="F169" s="2" t="n">
+        <v>738656120</v>
+      </c>
+      <c r="G169" s="2" t="n">
+        <v>738246060</v>
+      </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I169" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I169" s="2" t="inlineStr">
+        <is>
+          <t>Xujahurason mahallasi, Sugʻdiyona, 50 uy</t>
+        </is>
+      </c>
       <c r="J169" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz qishloq xo'jaligi kasb-hunar kolleji</t>
@@ -10651,15 +11269,21 @@
         </is>
       </c>
       <c r="F170" s="2" t="n">
-        <v>770683017</v>
-      </c>
-      <c r="G170" s="2" t="n"/>
+        <v>515384080</v>
+      </c>
+      <c r="G170" s="2" t="n">
+        <v>912849800</v>
+      </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I170" s="2" t="n"/>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>Oqsuv MFY, Nimgi qishloq, 38_uy</t>
+        </is>
+      </c>
       <c r="J170" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 46-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10718,10 +11342,14 @@
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I171" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
+        <is>
+          <t>Miraki mahallasi, Navoiy, 84 uy</t>
+        </is>
+      </c>
       <c r="J171" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 8-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10773,17 +11401,21 @@
         </is>
       </c>
       <c r="F172" s="2" t="n">
-        <v>933565022</v>
+        <v>335650220</v>
       </c>
       <c r="G172" s="2" t="n">
-        <v>910901627</v>
+        <v>109016270</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I172" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>Yomchi, Abdulqosim Firdavsiy, 134-uy</t>
+        </is>
+      </c>
       <c r="J172" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 23-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10835,15 +11467,21 @@
         </is>
       </c>
       <c r="F173" s="2" t="n">
-        <v>976188504</v>
-      </c>
-      <c r="G173" s="2" t="n"/>
+        <v>546564080</v>
+      </c>
+      <c r="G173" s="2" t="n">
+        <v>885040954</v>
+      </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Chiroqchi tumani</t>
-        </is>
-      </c>
-      <c r="I173" s="2" t="n"/>
+          <t>Qashqadaryo, Qamashi tumani</t>
+        </is>
+      </c>
+      <c r="I173" s="2" t="inlineStr">
+        <is>
+          <t>Yuksalish MFY, Olmazor, 124.0</t>
+        </is>
+      </c>
       <c r="J173" s="2" t="inlineStr">
         <is>
           <t>Chiroqchi tumani 70-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10894,14 +11532,22 @@
           <t>AE4246251</t>
         </is>
       </c>
-      <c r="F174" s="2" t="n"/>
-      <c r="G174" s="2" t="n"/>
+      <c r="F174" s="2" t="n">
+        <v>50305390</v>
+      </c>
+      <c r="G174" s="2" t="n">
+        <v>919510536</v>
+      </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I174" s="2" t="n"/>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>Nurafshon MFY, Kun botar, 101-uy</t>
+        </is>
+      </c>
       <c r="J174" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 36-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10953,17 +11599,21 @@
         </is>
       </c>
       <c r="F175" s="2" t="n">
-        <v>885581535</v>
+        <v>855815350</v>
       </c>
       <c r="G175" s="2" t="n">
-        <v>886331535</v>
+        <v>863315350</v>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I175" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>Yashil diyor mfy, Yashil diyor kuchasi, 118.0</t>
+        </is>
+      </c>
       <c r="J175" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 5-sonli umumiy o'rta ta'lim maktabi</t>
@@ -11015,17 +11665,21 @@
         </is>
       </c>
       <c r="F176" s="2" t="n">
-        <v>888191006</v>
+        <v>886061500</v>
       </c>
       <c r="G176" s="2" t="n">
-        <v>888606150</v>
+        <v>761500919</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I176" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>Meraki MFY, NAVOIY KÖCHASI, 48.0</t>
+        </is>
+      </c>
       <c r="J176" s="2" t="inlineStr">
         <is>
           <t>Miroq sport pedagogika kolleji</t>
@@ -11076,14 +11730,22 @@
           <t>AB6304158</t>
         </is>
       </c>
-      <c r="F177" s="2" t="n"/>
-      <c r="G177" s="2" t="n"/>
+      <c r="F177" s="2" t="n">
+        <v>505895877</v>
+      </c>
+      <c r="G177" s="2" t="n">
+        <v>871947276</v>
+      </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I177" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>Boston MFY, Kenagaz, 73- uy</t>
+        </is>
+      </c>
       <c r="J177" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz qurilish va maishiy texnikalar kasb-hunar kolleji</t>
@@ -11135,7 +11797,7 @@
         </is>
       </c>
       <c r="F178" s="2" t="n">
-        <v>931522577</v>
+        <v>315225770</v>
       </c>
       <c r="G178" s="2" t="n">
         <v>770867725</v>
@@ -11145,7 +11807,11 @@
           <t>Qashqadaryo, Yakkabog' tumani</t>
         </is>
       </c>
-      <c r="I178" s="2" t="n"/>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>Yashnabod MFY, Faravon kochasi, 223-uy</t>
+        </is>
+      </c>
       <c r="J178" s="2" t="inlineStr">
         <is>
           <t>Yakkabog' tumani 45-sonli umumiy o'rta ta'lim maktabi</t>
@@ -11197,17 +11863,21 @@
         </is>
       </c>
       <c r="F179" s="2" t="n">
-        <v>770209066</v>
+        <v>702090660</v>
       </c>
       <c r="G179" s="2" t="n">
-        <v>991638468</v>
+        <v>976175037</v>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I179" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>Ipak yuli, Ipak yuli, 128-uy</t>
+        </is>
+      </c>
       <c r="J179" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 15-sonli umumiy o'rta ta'lim maktabi</t>
@@ -11318,14 +11988,22 @@
           <t>AE4385291</t>
         </is>
       </c>
-      <c r="F181" s="2" t="n"/>
-      <c r="G181" s="2" t="n"/>
+      <c r="F181" s="2" t="n">
+        <v>938918590</v>
+      </c>
+      <c r="G181" s="2" t="n">
+        <v>976350269</v>
+      </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Qamashi tumani</t>
-        </is>
-      </c>
-      <c r="I181" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="inlineStr">
+        <is>
+          <t>Shamaton MFY, Yangiobod1, 111 uy</t>
+        </is>
+      </c>
       <c r="J181" s="2" t="inlineStr">
         <is>
           <t>Qamashi tumani 8-sonli umumiy o'rta ta'lim maktabi</t>
@@ -11377,17 +12055,21 @@
         </is>
       </c>
       <c r="F182" s="2" t="n">
+        <v>908810610</v>
+      </c>
+      <c r="G182" s="2" t="n">
         <v>908631674</v>
       </c>
-      <c r="G182" s="2" t="n">
-        <v>908810610</v>
-      </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I182" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahri</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>Fayzabod MFY, Quruvchilar ko'chasi, 73-uy</t>
+        </is>
+      </c>
       <c r="J182" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 15-sonli umumiy o'rta ta'lim maktabi</t>
@@ -11439,17 +12121,21 @@
         </is>
       </c>
       <c r="F183" s="2" t="n">
-        <v>773710028</v>
+        <v>737100280</v>
       </c>
       <c r="G183" s="2" t="n">
-        <v>956652882</v>
+        <v>566528820</v>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I183" s="2" t="n"/>
+      <c r="I183" s="2" t="inlineStr">
+        <is>
+          <t>Oqsuv MFY, Yoshlar kuchasi, 156-uy</t>
+        </is>
+      </c>
       <c r="J183" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 46-sonli umumiy o'rta ta'lim maktabi</t>
@@ -11501,17 +12187,21 @@
         </is>
       </c>
       <c r="F184" s="2" t="n">
-        <v>905181884</v>
+        <v>756130020</v>
       </c>
       <c r="G184" s="2" t="n">
-        <v>875613002</v>
+        <v>51818840</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I184" s="2" t="n"/>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>Ulugʻbek MFY, Urigzor koʻchasi, 23 -uy</t>
+        </is>
+      </c>
       <c r="J184" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 32-sonli umumiy o'rta ta'lim maktabi</t>

</xml_diff>

<commit_message>
fix: Word va Excel eksport jurnallaridagi buzilish xatoliklari to'liq bartaraf etildi
</commit_message>
<xml_diff>
--- a/hisobotlar/qabul/QABUL - 2026.xlsx
+++ b/hisobotlar/qabul/QABUL - 2026.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:N184"/>
+  <dimension ref="A3:N183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.14" customWidth="1" min="1" max="1"/>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>884808270</v>
+        <v>888480827</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>978550581</v>
@@ -617,10 +617,10 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>24337740</v>
+        <v>902433774</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>858881870</v>
+        <v>885888187</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -683,14 +683,14 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>536726020</v>
+        <v>953672602</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>906161560</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -815,14 +815,14 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>121770090</v>
+        <v>912177009</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>65620200</v>
+        <v>914606562</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -881,14 +881,14 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>749526080</v>
+        <v>874952608</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>973873803</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
+          <t>Qashqadaryo, Kitob tumani sevaz shaharchasi</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1013,14 +1013,14 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>838893260</v>
+        <v>883889326</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>968513210</v>
+        <v>996851321</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tuman</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1079,14 +1079,14 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>775119810</v>
+        <v>877511981</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>919490180</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1145,14 +1145,14 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>90713110</v>
+        <v>509071311</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>973808965</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>6673090</v>
+        <v>700667309</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>703902308</v>
@@ -1277,19 +1277,19 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>756108880</v>
+        <v>875610888</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>936031585</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Duxchi MFY, Duxchi qishlog'i, 148.0</t>
+          <t>Duxchi MFY, Duxchi qishlog'i, 148-uy</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1343,14 +1343,14 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>107075010</v>
+        <v>910707501</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>86982090</v>
+        <v>908698209</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1409,14 +1409,14 @@
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>122400180</v>
+        <v>912240018</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>912240018</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1475,10 +1475,10 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>3431310</v>
+        <v>700343131</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>3431310</v>
+        <v>700343131</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Guluston, Guluston, 4.0</t>
+          <t>Guluston, Guluston, 4-uy</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1541,14 +1541,14 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>706298900</v>
+        <v>770629890</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>973196260</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1609,7 +1609,9 @@
       <c r="F20" s="2" t="n">
         <v>976190215</v>
       </c>
-      <c r="G20" s="2" t="n"/>
+      <c r="G20" s="2" t="n">
+        <v>887311969</v>
+      </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Chiroqchi tumani</t>
@@ -1678,7 +1680,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, shahrizabz shahar</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1737,14 +1739,14 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>701026210</v>
+        <v>870102621</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>977011783</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
+          <t>Qashqadaryo viloyati Kitob tumani</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1803,7 +1805,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>756815080</v>
+        <v>875681508</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>885857068</v>
@@ -1869,17 +1871,21 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>973350582</v>
+        <v>978635082</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>978635082</v>
+        <v>973550582</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I24" s="2" t="n"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Saroy MFY, Yangiqishloq, 44-uy</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 47-sonli umumiy o'rta ta'lim maktabi</t>
@@ -1931,14 +1937,14 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>811510310</v>
+        <v>881151031</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>881840585</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1997,15 +2003,21 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
+        <v>778641917</v>
+      </c>
+      <c r="G26" s="2" t="n">
         <v>912174355</v>
       </c>
-      <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Turon MFY, Yangi obod, 62-uy</t>
+        </is>
+      </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 14-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2060,14 +2072,18 @@
         <v>918112208</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>918151309</v>
+        <v>918172073</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I27" s="2" t="n"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Saroy MFY, Saroy koʻchasi, 17-uy</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 47-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2119,14 +2135,14 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>808801240</v>
+        <v>880880124</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>156130020</v>
+        <v>915613002</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
+          <t>Qashqadaryo, Kotob tumani</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2185,19 +2201,19 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>184403080</v>
+        <v>918440308</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>195942150</v>
+        <v>919594215</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Qiziltepa tumani</t>
+          <t>Qashqadaryo, Qizil tepa</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Yuksalish mfy, Roxat koʻchasi, 44.0</t>
+          <t>Yuksalish mfy, Roxat koʻchasi, 44-uy</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2251,10 +2267,10 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>721302400</v>
+        <v>872130240</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>861885800</v>
+        <v>886188580</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -2263,7 +2279,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Palandara MFY, Oftobroʻya qishlogʻi, 35.0</t>
+          <t>Palandara MFY, Oftobroʻya qishlogʻi, 35-uy</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2320,11 +2336,11 @@
         <v>776070824</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>739901790</v>
+        <v>873990179</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2448,7 +2464,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2567,10 +2583,10 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>87851050</v>
+        <v>908785105</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>163976850</v>
+        <v>916397685</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -2633,19 +2649,19 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>505054080</v>
+        <v>950505408</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>906262080</v>
+        <v>990626208</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Qamashi tumani</t>
+          <t>Qashqadaryo, Qamashi</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Yuksalish MFY, Olmazor, 183.0</t>
+          <t>Yuksalish MFY, Olmazor, 183-uy</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2699,14 +2715,14 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>163545560</v>
+        <v>916354556</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>953332960</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2832,7 +2848,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shaxrisabz tumani</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2890,14 +2906,22 @@
           <t>AE4233482</t>
         </is>
       </c>
-      <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
+      <c r="F40" s="2" t="n">
+        <v>500026078</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>500026078</v>
+      </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I40" s="2" t="n"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Qashqadaryo MFY, Minjir qishlogʻi, 51-uy</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 78-sonli umumiy o'rta ta'lim maktabi</t>
@@ -2956,7 +2980,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -3015,10 +3039,10 @@
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>794119200</v>
+        <v>879411920</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>961522720</v>
+        <v>996152272</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -3027,7 +3051,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Zarafshon MFY, Yangiobod shaharchasi, 432.0</t>
+          <t>Zarafshon MFY, Yangiobod shaharchasi, 432-uy</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3081,19 +3105,19 @@
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>886899080</v>
+        <v>883367774</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>577011690</v>
+        <v>907163142</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Shanbe MFY, Shabboda, 35 -uy</t>
+          <t>Do'stlik MFY, Bunyodkor ko'chasi, 62/16-uy</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3147,10 +3171,10 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>801158190</v>
+        <v>880115819</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>505870874</v>
+        <v>874650587</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -3213,14 +3237,14 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>146492280</v>
+        <v>914649228</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>886015200</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shaxrsabz shahar</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -3279,7 +3303,7 @@
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>593907050</v>
+        <v>959390705</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>991437903</v>
@@ -3345,14 +3369,14 @@
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>736908720</v>
+        <v>873690872</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>806692720</v>
+        <v>880669272</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -3414,16 +3438,16 @@
         <v>334948423</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>494842333</v>
+        <v>334948423</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>G'arov, G'arov kuchasi, 84.0</t>
+          <t>G'arov, G'arov kuchasi, 84-uy</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -3477,10 +3501,10 @@
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>7206140</v>
+        <v>700720614</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>577415640</v>
+        <v>957741564</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -3543,10 +3567,10 @@
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>700880280</v>
+        <v>970088028</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>880280880</v>
+        <v>880088028</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -3612,14 +3636,18 @@
         <v>771219093</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>889770693</v>
+        <v>992019274</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I51" s="2" t="n"/>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Ayoqchi MFY, Qovchin qishlogʻi, 92uy</t>
+        </is>
+      </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 45-sonli umumiy o'rta ta'lim maktabi</t>
@@ -3729,10 +3757,10 @@
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>407901060</v>
+        <v>940790106</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>351375740</v>
+        <v>935137574</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
@@ -3797,13 +3825,19 @@
       <c r="F54" s="2" t="n">
         <v>917090876</v>
       </c>
-      <c r="G54" s="2" t="n"/>
+      <c r="G54" s="2" t="n">
+        <v>918127697</v>
+      </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Yakkabog' tumani</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="n"/>
+          <t>Qashqadaryo, Yakkabogʻ tumani</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Tatar MFY, Yangi hayot koʻchasi, 49_uy</t>
+        </is>
+      </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
           <t>Yakkabog' tumani 25-sonli umumiy o'rta ta'lim maktabi</t>
@@ -3862,7 +3896,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Yakkabog' tumani</t>
+          <t>Qashqadaryo, Yakkabogʻ tumani</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -4045,14 +4079,14 @@
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>593992050</v>
+        <v>959399205</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>523327660</v>
+        <v>952332766</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -4111,14 +4145,14 @@
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>45042400</v>
+        <v>504504240</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>939034744</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo viloyati</t>
+          <t>Qashqadaryo, Qashqadaryo tumani</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -4355,14 +4389,14 @@
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>780066370</v>
+        <v>878006637</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>970012780</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -4424,11 +4458,11 @@
         <v>772131924</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>548408291</v>
+        <v>915484082</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -4494,12 +4528,12 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Oq Oltin MFY, Al-Xorazmiy koʼchasi, 212-uy</t>
+          <t>Oq Oltin MFY, Al- Xorazmiy, 212-uy</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -4622,12 +4656,12 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrizabz tumani</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Turon MFY, Turon koʻchasi, 52.0</t>
+          <t>Turon MFY, Turon koʻchasi, 52-uy</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -4681,14 +4715,14 @@
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>195957710</v>
+        <v>919595771</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>919595771</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -4747,7 +4781,7 @@
         </is>
       </c>
       <c r="F69" s="2" t="n">
-        <v>806326080</v>
+        <v>880632608</v>
       </c>
       <c r="G69" s="2" t="n">
         <v>973360140</v>
@@ -4881,7 +4915,11 @@
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="I71" s="2" t="n"/>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Bunyodkor, Alpomish, 13-uy</t>
+        </is>
+      </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 7-sonli umumiy o'rta ta'lim maktabi</t>
@@ -4933,10 +4971,10 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>47809270</v>
+        <v>704780927</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>305783230</v>
+        <v>330578323</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -4999,19 +5037,19 @@
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>850207030</v>
+        <v>885020703</v>
       </c>
       <c r="G73" s="2" t="n">
         <v>880037679</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Yakkabog' tumani</t>
+          <t>Qashqadaryo, Yakkabogʼ</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>Chagʼatoy, Yuq, 76.0</t>
+          <t>Chagʼatoy, Yuq, 76-uy</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -5072,12 +5110,12 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabiz tumani</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>Sanam MFY, Uzumzor kochasi, 60.0</t>
+          <t>Sanam MFY, Uzumzor kochasi, 60-uy</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -5131,14 +5169,14 @@
         </is>
       </c>
       <c r="F75" s="2" t="n">
-        <v>558388580</v>
+        <v>955838858</v>
       </c>
       <c r="G75" s="2" t="n">
         <v>916417532</v>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
@@ -5204,7 +5242,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -5263,14 +5301,14 @@
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>876113100</v>
+        <v>887611310</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>738982040</v>
+        <v>973898204</v>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
+          <t>Qashqadaryo, Китабский район</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -5398,12 +5436,12 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Китоб</t>
+          <t>Qashqadaryo, китоб</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>китоб МФЯ, гулустон кучаси, 90.0</t>
+          <t>китоб МФЯ, гулустон кучаси, 90-uy</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -5457,14 +5495,14 @@
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>898183800</v>
+        <v>889818380</v>
       </c>
       <c r="G80" s="2" t="n">
         <v>883861712</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
@@ -5523,10 +5561,10 @@
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>722542080</v>
+        <v>772254208</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>994513820</v>
+        <v>999451382</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -5589,7 +5627,7 @@
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>862338080</v>
+        <v>886233808</v>
       </c>
       <c r="G82" s="2" t="n">
         <v>770216705</v>
@@ -5655,19 +5693,19 @@
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>514708250</v>
+        <v>951470825</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>224730951</v>
+        <v>997422473</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Yakkabog' tumani</t>
+          <t>Qashqadaryo, Yakkabog'</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>Kenguzar MFY, Chig'atoy, 6.0</t>
+          <t>Kenguzar MFY, Chig'atoy, 6-uy</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -5721,10 +5759,10 @@
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>804102270</v>
+        <v>880410227</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>817080810</v>
+        <v>881708081</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -5733,7 +5771,7 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>Xoji MFY, Uzunqir kuchasi, 106.0</t>
+          <t>Xoji MFY, Uzunqir kuchasi, 106-uy</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -5849,19 +5887,19 @@
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>913125080</v>
+        <v>991312508</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>760782870</v>
+        <v>886078287</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>Kichik novqat mfy, Soyboʻyi koʻchasi, 04</t>
+          <t>Maktobod mfy, Soyboʻyi koʻchasi, 4-uy</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -5915,10 +5953,10 @@
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>33187080</v>
+        <v>703318708</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>11906860</v>
+        <v>701190686</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -5927,7 +5965,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>Quruq soy MFY, Buzovut qishlogʻi, 111-uy</t>
+          <t>Quruqsoy MFY, Buzovut qishlogʻi, 111-uy</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -5981,17 +6019,21 @@
         </is>
       </c>
       <c r="F88" s="2" t="n">
+        <v>879266108</v>
+      </c>
+      <c r="G88" s="2" t="n">
         <v>919483879</v>
       </c>
-      <c r="G88" s="2" t="n">
-        <v>885967179</v>
-      </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I88" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>Nomozgoh MFY, Taragʻay Bahodir, 2.31-uy</t>
+        </is>
+      </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 13-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6043,14 +6085,14 @@
         </is>
       </c>
       <c r="F89" s="2" t="n">
-        <v>759109180</v>
+        <v>875910918</v>
       </c>
       <c r="G89" s="2" t="n">
         <v>885660802</v>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shaxrisabz shahri</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
@@ -6109,14 +6151,14 @@
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>763104770</v>
+        <v>876310477</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>732104770</v>
+        <v>873210477</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
@@ -6182,12 +6224,12 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Yakkabog' tumani</t>
+          <t>Qashqadaryo, Yakkabogʻ tumani</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>Alakuylak MFY, Hamid Olimjon koʻchasi, 55.0</t>
+          <t>Alakuylak MFY, Hamid Olimjon koʻchasi, 55-uy</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -6369,17 +6411,21 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>910054908</v>
+        <v>882054908</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>935533351</v>
+        <v>887533351</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I94" s="2" t="n"/>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>Katlos MFY, Bogʻiston kòchasi, 28-uy</t>
+        </is>
+      </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 61-sonli umumiy o'rta ta'lim maktabi</t>
@@ -6431,19 +6477,19 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>834030080</v>
+        <v>883403008</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>952647090</v>
+        <v>995264709</v>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>Guliston MFY, Qoʻshtepa kòchasi, 329.0</t>
+          <t>Guliston MFY, Qoʻshtepa kòchasi, 329-uy</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -6497,7 +6543,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>1114090</v>
+        <v>500111409</v>
       </c>
       <c r="G96" s="2" t="n">
         <v>973891174</v>
@@ -6563,10 +6609,10 @@
         </is>
       </c>
       <c r="F97" s="2" t="n">
-        <v>44036660</v>
+        <v>904403666</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>122477210</v>
+        <v>912247721</v>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
@@ -6641,7 +6687,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>Iskana MFY, Uchtepalik, 52.0</t>
+          <t>Iskana MFY, Uchtepalik, 52-uy</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -6695,14 +6741,14 @@
         </is>
       </c>
       <c r="F99" s="2" t="n">
-        <v>58999480</v>
+        <v>505899948</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>73473860</v>
+        <v>507347386</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
+          <t>Qashqadaryo, Boshchil qishlog'i</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
@@ -6764,7 +6810,7 @@
         <v>874637908</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>107095790</v>
+        <v>910709579</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -6827,14 +6873,14 @@
         </is>
       </c>
       <c r="F101" s="2" t="n">
-        <v>916820820</v>
+        <v>991682082</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>916820820</v>
+        <v>991682082</v>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Yakkabog' tumani</t>
+          <t>Qashqadaryo, Yakkabogʻ tumani</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
@@ -6893,10 +6939,10 @@
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>88412080</v>
+        <v>908841208</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>195727170</v>
+        <v>919572717</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -6905,7 +6951,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>Uluğbek MFY, Mirzo Tursunzoda kòchasi, 49.0</t>
+          <t>Uluğbek MFY, Mirzo Tursunzoda kòchasi, 49-uy</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -7024,14 +7070,22 @@
           <t>AD9484395</t>
         </is>
       </c>
-      <c r="F104" s="2" t="n"/>
-      <c r="G104" s="2" t="n"/>
+      <c r="F104" s="2" t="n">
+        <v>938041814</v>
+      </c>
+      <c r="G104" s="2" t="n">
+        <v>973858369</v>
+      </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="I104" s="2" t="n"/>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>Abziyat MFY, Hidoyat ko’chasi, 1-uy</t>
+        </is>
+      </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 22-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7083,19 +7137,19 @@
         </is>
       </c>
       <c r="F105" s="2" t="n">
-        <v>87802800</v>
+        <v>908780280</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>526948780</v>
+        <v>952694878</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tuman</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>Xitoy MFY, Besh chinor, 65.0</t>
+          <t>Xitoy MFY, Besh chinor, 65-uy</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -7149,14 +7203,14 @@
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>833677740</v>
+        <v>883367774</v>
       </c>
       <c r="G106" s="2" t="n">
         <v>907163142</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
@@ -7275,7 +7329,7 @@
         </is>
       </c>
       <c r="F108" s="2" t="n">
-        <v>702902740</v>
+        <v>770290274</v>
       </c>
       <c r="G108" s="2" t="n">
         <v>882633833</v>
@@ -7287,7 +7341,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>Guliston MFY, Qo'shtepa mahallasi, 75.0</t>
+          <t>Guliston MFY, Qo'shtepa mahallasi, 75-uy</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -7341,10 +7395,10 @@
         </is>
       </c>
       <c r="F109" s="2" t="n">
-        <v>858727010</v>
+        <v>885872701</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>68720885</v>
+        <v>884906872</v>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
@@ -7407,10 +7461,10 @@
         </is>
       </c>
       <c r="F110" s="2" t="n">
-        <v>711603030</v>
+        <v>871160303</v>
       </c>
       <c r="G110" s="2" t="n">
-        <v>711603030</v>
+        <v>871160303</v>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
@@ -7539,14 +7593,14 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>793403010</v>
+        <v>879340301</v>
       </c>
       <c r="G112" s="2" t="n">
-        <v>872288840</v>
+        <v>887228884</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr">
@@ -7605,17 +7659,21 @@
         </is>
       </c>
       <c r="F113" s="2" t="n">
-        <v>976760905</v>
+        <v>977874795</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>876317371</v>
+        <v>976979592</v>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
-        </is>
-      </c>
-      <c r="I113" s="2" t="n"/>
+          <t>Qashqadaryo, Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>Chiroqchi MFY, Elabot kuchasi, 227-uy</t>
+        </is>
+      </c>
       <c r="J113" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 19-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7670,14 +7728,18 @@
         <v>333801121</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>880096166</v>
+        <v>935629405</v>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I114" s="2" t="n"/>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>Nurali MFY, Nurali qishlogi, 75-uy</t>
+        </is>
+      </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 3-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7729,10 +7791,10 @@
         </is>
       </c>
       <c r="F115" s="2" t="n">
-        <v>68161770</v>
+        <v>706816177</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>961660883</v>
+        <v>880096166</v>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
@@ -7741,7 +7803,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>Xalqlar do'stligi MFY, Qashqadaryo2, 65.0</t>
+          <t>Xalqlar do'stligi MFY, Qashqadaryo2, 65-uy</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -7798,14 +7860,18 @@
         <v>887291401</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>976198484</v>
+        <v>973878737</v>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="I116" s="2" t="n"/>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>Qumqishloq MFY, Hoji koʻchasi, 2-uy</t>
+        </is>
+      </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 15-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7857,10 +7923,10 @@
         </is>
       </c>
       <c r="F117" s="2" t="n">
-        <v>311580830</v>
+        <v>331158083</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>883800339</v>
+        <v>976188380</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -7923,15 +7989,21 @@
         </is>
       </c>
       <c r="F118" s="2" t="n">
-        <v>918715737</v>
-      </c>
-      <c r="G118" s="2" t="n"/>
+        <v>770069149</v>
+      </c>
+      <c r="G118" s="2" t="n">
+        <v>909604580</v>
+      </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
-        </is>
-      </c>
-      <c r="I118" s="2" t="n"/>
+          <t>Qashqadaryo, Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>Taragʻay MFY, Taragʻay, Yuq</t>
+        </is>
+      </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 109-sonli umumiy o'rta ta'lim maktabi</t>
@@ -7983,7 +8055,7 @@
         </is>
       </c>
       <c r="F119" s="2" t="n">
-        <v>338905030</v>
+        <v>333890503</v>
       </c>
       <c r="G119" s="2" t="n">
         <v>949791283</v>
@@ -8111,14 +8183,14 @@
         </is>
       </c>
       <c r="F121" s="2" t="n">
-        <v>743217070</v>
+        <v>774321707</v>
       </c>
       <c r="G121" s="2" t="n">
-        <v>561635090</v>
+        <v>956163509</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I121" s="2" t="inlineStr">
@@ -8177,14 +8249,14 @@
         </is>
       </c>
       <c r="F122" s="2" t="n">
-        <v>830902280</v>
+        <v>883090228</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>800578080</v>
+        <v>880057808</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I122" s="2" t="inlineStr">
@@ -8243,7 +8315,7 @@
         </is>
       </c>
       <c r="F123" s="2" t="n">
-        <v>840204080</v>
+        <v>884020408</v>
       </c>
       <c r="G123" s="2" t="n">
         <v>990630419</v>
@@ -8371,19 +8443,19 @@
         </is>
       </c>
       <c r="F125" s="2" t="n">
-        <v>762945080</v>
+        <v>957401981</v>
       </c>
       <c r="G125" s="2" t="n">
-        <v>873819820</v>
+        <v>957401981</v>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>Toʻdamaydon, Fidokor, 92.0</t>
+          <t>Toʻdamaydon, Fidokor, 92-uy</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -8437,19 +8509,19 @@
         </is>
       </c>
       <c r="F126" s="2" t="n">
-        <v>818311670</v>
+        <v>876295108</v>
       </c>
       <c r="G126" s="2" t="n">
-        <v>183116787</v>
+        <v>881831167</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
+          <t>Qashqadaryo, Kitob</t>
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>Iskana MFY, Iskana ko'chasi, 40-uy</t>
+          <t>Iksana MFY, Iskana qishloqi, 40-uy</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -8503,7 +8575,7 @@
         </is>
       </c>
       <c r="F127" s="2" t="n">
-        <v>793476080</v>
+        <v>879347608</v>
       </c>
       <c r="G127" s="2" t="n">
         <v>914564661</v>
@@ -8515,7 +8587,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>BektimirMFY, Yoshlar kuchasi, 27.0</t>
+          <t>BektimirMFY, Yoshlar kuchasi, 27-uy</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -8569,15 +8641,21 @@
         </is>
       </c>
       <c r="F128" s="2" t="n">
+        <v>778181856</v>
+      </c>
+      <c r="G128" s="2" t="n">
         <v>976180259</v>
       </c>
-      <c r="G128" s="2" t="n"/>
       <c r="H128" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I128" s="2" t="n"/>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>Beshariq MFY, Mehrobod, 45-uy</t>
+        </is>
+      </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 6-sonli umumiy o'rta ta'lim maktabi</t>
@@ -8632,7 +8710,7 @@
         <v>978527404</v>
       </c>
       <c r="G129" s="2" t="n">
-        <v>785274040</v>
+        <v>978527404</v>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
@@ -8641,7 +8719,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>Katlos mfy, Obigarm kuchasi, 89.0</t>
+          <t>Katlos mfy, Obigarm kuchasi, 89-uy</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -8695,10 +8773,10 @@
         </is>
       </c>
       <c r="F130" s="2" t="n">
-        <v>460344070</v>
+        <v>946034407</v>
       </c>
       <c r="G130" s="2" t="n">
-        <v>30150780</v>
+        <v>903015078</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -8764,14 +8842,18 @@
         <v>701206508</v>
       </c>
       <c r="G131" s="2" t="n">
-        <v>995698112</v>
+        <v>995688112</v>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
           <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
-      <c r="I131" s="2" t="n"/>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>Oqsuv MFY, Nimgi qishloq, 152-uy</t>
+        </is>
+      </c>
       <c r="J131" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 46-sonli umumiy o'rta ta'lim maktabi</t>
@@ -8889,19 +8971,19 @@
         </is>
       </c>
       <c r="F133" s="2" t="n">
-        <v>881796080</v>
+        <v>888179608</v>
       </c>
       <c r="G133" s="2" t="n">
-        <v>530860888</v>
+        <v>950753086</v>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>Miraki mfy, Navoiy ko'chasi, 68.0</t>
+          <t>Miraki mfy, Navoiy ko'chasi, 68-uy</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -8955,17 +9037,21 @@
         </is>
       </c>
       <c r="F134" s="2" t="n">
-        <v>701885432</v>
+        <v>778380748</v>
       </c>
       <c r="G134" s="2" t="n">
         <v>958050186</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
-        </is>
-      </c>
-      <c r="I134" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrissbz tumani</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>Zangi, Keldihayot koʻchasi 290, 290-uy</t>
+        </is>
+      </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 1-son politexnikumi</t>
@@ -9019,13 +9105,19 @@
       <c r="F135" s="2" t="n">
         <v>919571858</v>
       </c>
-      <c r="G135" s="2" t="n"/>
+      <c r="G135" s="2" t="n">
+        <v>970340530</v>
+      </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
-        </is>
-      </c>
-      <c r="I135" s="2" t="n"/>
+          <t>Qashqadaryo, Kitob tuman</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>Hamid Olimjon, Zilol buloq, 17-uy</t>
+        </is>
+      </c>
       <c r="J135" s="2" t="inlineStr">
         <is>
           <t>Kitob tumani 29-sonli umumiy o'rta ta'lim maktabi</t>
@@ -9077,10 +9169,10 @@
         </is>
       </c>
       <c r="F136" s="2" t="n">
-        <v>107102830</v>
+        <v>910710283</v>
       </c>
       <c r="G136" s="2" t="n">
-        <v>107102830</v>
+        <v>910710283</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -9089,7 +9181,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>Hamid Olimjon MFY, Amir Temur, 69.0</t>
+          <t>Hamid Olimjon MFY, Amir Temur, 69-uy</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -9143,10 +9235,10 @@
         </is>
       </c>
       <c r="F137" s="2" t="n">
-        <v>738899780</v>
+        <v>973889978</v>
       </c>
       <c r="G137" s="2" t="n">
-        <v>755860880</v>
+        <v>908775586</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
@@ -9209,17 +9301,21 @@
         </is>
       </c>
       <c r="F138" s="2" t="n">
-        <v>919491627</v>
+        <v>900698998</v>
       </c>
       <c r="G138" s="2" t="n">
         <v>900698998</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I138" s="2" t="n"/>
+          <t>Qashqadaryo, Shaxresabiz tumani</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>Quchi MFY, Quchi kuchasi, 56-uy</t>
+        </is>
+      </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz agrosanoat kasb-hunar kolleji</t>
@@ -9329,19 +9425,19 @@
         </is>
       </c>
       <c r="F140" s="2" t="n">
-        <v>910608100</v>
+        <v>991060810</v>
       </c>
       <c r="G140" s="2" t="n">
-        <v>781800701</v>
+        <v>955278180</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>Sayyod MFY, Obod mahallasi, 13.0</t>
+          <t>Sayyod MFY, Obod mahallasi, 13-uy</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -9395,10 +9491,10 @@
         </is>
       </c>
       <c r="F141" s="2" t="n">
-        <v>796563080</v>
+        <v>779656308</v>
       </c>
       <c r="G141" s="2" t="n">
-        <v>713906770</v>
+        <v>971390677</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -9407,7 +9503,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>Surum mahallasi, Sokin koʻchasi, 66.0</t>
+          <t>Surum mahallasi, Sokin koʻchasi, 66-uy</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -9461,7 +9557,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>180216700</v>
+        <v>918021670</v>
       </c>
       <c r="G142" s="2" t="n">
         <v>919614037</v>
@@ -9527,19 +9623,19 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>86424710</v>
+        <v>908642471</v>
       </c>
       <c r="G143" s="2" t="n">
-        <v>194964710</v>
+        <v>919496471</v>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>Dustlik mahallasi, Bunyodkor kuchasi, 97.0</t>
+          <t>Dustlik MFY, Bunyodkor kuchasi, 97-uy</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -9593,14 +9689,14 @@
         </is>
       </c>
       <c r="F144" s="2" t="n">
-        <v>196008140</v>
+        <v>919600814</v>
       </c>
       <c r="G144" s="2" t="n">
         <v>912250767</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I144" s="2" t="inlineStr">
@@ -9659,10 +9755,10 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>780982300</v>
+        <v>778098130</v>
       </c>
       <c r="G145" s="2" t="n">
-        <v>956586810</v>
+        <v>995658681</v>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
@@ -9671,7 +9767,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>Navbahor MFY, Yangi jilisuv qishlogʻi, 99 uy</t>
+          <t>Jilisuv MFY, Yangi Jilisuv, 99-uy</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -9725,10 +9821,10 @@
         </is>
       </c>
       <c r="F146" s="2" t="n">
-        <v>780981300</v>
+        <v>778098230</v>
       </c>
       <c r="G146" s="2" t="n">
-        <v>956586810</v>
+        <v>995658681</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
@@ -9737,7 +9833,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>Jilisuv MFY, Yangi Jilisuv, 99.0</t>
+          <t>Navbahor MFY, Yangi jilisuv qishlogʻi, 99 uy</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -9791,14 +9887,14 @@
         </is>
       </c>
       <c r="F147" s="2" t="n">
-        <v>700046080</v>
+        <v>870004608</v>
       </c>
       <c r="G147" s="2" t="n">
         <v>771088048</v>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I147" s="2" t="inlineStr">
@@ -9860,11 +9956,11 @@
         <v>995590930</v>
       </c>
       <c r="G148" s="2" t="n">
-        <v>518201950</v>
+        <v>951820195</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Yakkabog' tumani</t>
+          <t>Qashqadaryo, Yakkabogʻ tumani</t>
         </is>
       </c>
       <c r="I148" s="2" t="inlineStr">
@@ -9923,7 +10019,7 @@
         </is>
       </c>
       <c r="F149" s="2" t="n">
-        <v>48913000</v>
+        <v>904891300</v>
       </c>
       <c r="G149" s="2" t="n">
         <v>908708827</v>
@@ -9989,10 +10085,10 @@
         </is>
       </c>
       <c r="F150" s="2" t="n">
-        <v>189804950</v>
+        <v>918980495</v>
       </c>
       <c r="G150" s="2" t="n">
-        <v>88308650</v>
+        <v>908830865</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -10128,12 +10224,12 @@
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shaxar</t>
         </is>
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>Kesh, Kalokon, 73 uy</t>
+          <t>Kesh mahalas, Kalakon kuchas, 73-uy</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -10194,7 +10290,7 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr">
@@ -10253,7 +10349,7 @@
         </is>
       </c>
       <c r="F154" s="2" t="n">
-        <v>878860420</v>
+        <v>887886042</v>
       </c>
       <c r="G154" s="2" t="n">
         <v>916383271</v>
@@ -10319,19 +10415,19 @@
         </is>
       </c>
       <c r="F155" s="2" t="n">
-        <v>198815080</v>
+        <v>919881508</v>
       </c>
       <c r="G155" s="2" t="n">
-        <v>904810912</v>
+        <v>912237520</v>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Yakkabog' tumani</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>Darxon MFY, Eshonguzar, 52-uy</t>
+          <t>Darxon MFY, Eshonguzar kôchasi, 52-uy</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -10384,14 +10480,22 @@
           <t>AC2430931</t>
         </is>
       </c>
-      <c r="F156" s="2" t="n"/>
-      <c r="G156" s="2" t="n"/>
+      <c r="F156" s="2" t="n">
+        <v>915626577</v>
+      </c>
+      <c r="G156" s="2" t="n">
+        <v>918127080</v>
+      </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I156" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz Shahar</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>Farovon, Farovon kuchasi, 14-uy</t>
+        </is>
+      </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 14-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10443,17 +10547,21 @@
         </is>
       </c>
       <c r="F157" s="2" t="n">
+        <v>778108280</v>
+      </c>
+      <c r="G157" s="2" t="n">
         <v>919524344</v>
       </c>
-      <c r="G157" s="2" t="n">
-        <v>904422247</v>
-      </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="I157" s="2" t="n"/>
+          <t>Qashqadaryo, Shahrisabz shaxar</t>
+        </is>
+      </c>
+      <c r="I157" s="2" t="inlineStr">
+        <is>
+          <t>Sinabog MFY, oqshom, 112-uy</t>
+        </is>
+      </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz tumani 23-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10505,14 +10613,14 @@
         </is>
       </c>
       <c r="F158" s="2" t="n">
-        <v>502028130</v>
+        <v>950202813</v>
       </c>
       <c r="G158" s="2" t="n">
-        <v>727528130</v>
+        <v>772752813</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shaxrisabiz shahar</t>
         </is>
       </c>
       <c r="I158" s="2" t="inlineStr">
@@ -10633,10 +10741,10 @@
         </is>
       </c>
       <c r="F160" s="2" t="n">
-        <v>967399290</v>
+        <v>996739929</v>
       </c>
       <c r="G160" s="2" t="n">
-        <v>967399290</v>
+        <v>996739929</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
@@ -10645,7 +10753,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>Katlos MFY, Oshqon kuchasi, 69-uy</t>
+          <t>Katlos MFY, Oshqon, 69-uy</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -10759,7 +10867,7 @@
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>329607080</v>
+        <v>332960708</v>
       </c>
       <c r="G162" s="2" t="n">
         <v>881360926</v>
@@ -10771,7 +10879,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>Sariosiyo MFY, Chinorlik ko'chasi, 14.0</t>
+          <t>Sariosiyo MFY, Chinorlik koʻchasi, 14-uy</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -10825,10 +10933,10 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>873261110</v>
+        <v>887326111</v>
       </c>
       <c r="G163" s="2" t="n">
-        <v>768830906</v>
+        <v>916176883</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
@@ -10837,7 +10945,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>Ulugʻbek MFY, Qizil darvoza kuchasi, 116.0</t>
+          <t>Ulugʻbek MFY, Qizil darvoza kuchasi, 116-uy</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -10891,17 +10999,21 @@
         </is>
       </c>
       <c r="F164" s="2" t="n">
-        <v>912171430</v>
+        <v>882446808</v>
       </c>
       <c r="G164" s="2" t="n">
-        <v>941343403</v>
+        <v>880271582</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
-        </is>
-      </c>
-      <c r="I164" s="2" t="n"/>
+          <t>Qashqadaryo, Chiroqchi</t>
+        </is>
+      </c>
+      <c r="I164" s="2" t="inlineStr">
+        <is>
+          <t>Hamid olimjon MFY, Haytkul, 115-uy</t>
+        </is>
+      </c>
       <c r="J164" s="2" t="inlineStr">
         <is>
           <t>Shahrisabz shahri 35-sonli umumiy o'rta ta'lim maktabi</t>
@@ -10953,14 +11065,14 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>771601300</v>
+        <v>877160130</v>
       </c>
       <c r="G165" s="2" t="n">
-        <v>838879120</v>
+        <v>883887912</v>
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I165" s="2" t="inlineStr">
@@ -11079,14 +11191,14 @@
         </is>
       </c>
       <c r="F167" s="2" t="n">
-        <v>765900270</v>
+        <v>876590027</v>
       </c>
       <c r="G167" s="2" t="n">
-        <v>707908680</v>
+        <v>870790868</v>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahrar</t>
         </is>
       </c>
       <c r="I167" s="2" t="inlineStr">
@@ -11203,19 +11315,19 @@
         </is>
       </c>
       <c r="F169" s="2" t="n">
-        <v>738656120</v>
+        <v>973865612</v>
       </c>
       <c r="G169" s="2" t="n">
-        <v>738246060</v>
+        <v>973824606</v>
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>Xujahurason mahallasi, Sugʻdiyona, 50 uy</t>
+          <t>Xujahurason mahalla, Sugʻdiyona, 50-uy</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -11269,10 +11381,10 @@
         </is>
       </c>
       <c r="F170" s="2" t="n">
-        <v>515384080</v>
+        <v>951538408</v>
       </c>
       <c r="G170" s="2" t="n">
-        <v>912849800</v>
+        <v>991284980</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -11281,7 +11393,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>Oqsuv MFY, Nimgi qishloq, 38_uy</t>
+          <t>Oqsuv, Nimgi qishloq, 38-uy</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -11342,12 +11454,12 @@
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Miraki</t>
         </is>
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>Miraki mahallasi, Navoiy, 84 uy</t>
+          <t>Alisher Navoiy, Navoiy kuchasi, 84 uy</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -11401,19 +11513,19 @@
         </is>
       </c>
       <c r="F172" s="2" t="n">
-        <v>335650220</v>
+        <v>933565022</v>
       </c>
       <c r="G172" s="2" t="n">
-        <v>109016270</v>
+        <v>910901627</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>Yomchi, Abdulqosim Firdavsiy, 134-uy</t>
+          <t>Q9oʻrgʻon tepa MFY, Abdulqodimfirdavsiy koʻchasi, 134-uy</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -11467,10 +11579,10 @@
         </is>
       </c>
       <c r="F173" s="2" t="n">
-        <v>546564080</v>
+        <v>954656408</v>
       </c>
       <c r="G173" s="2" t="n">
-        <v>885040954</v>
+        <v>976188504</v>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
@@ -11479,7 +11591,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>Yuksalish MFY, Olmazor, 124.0</t>
+          <t>Yuksalish MFY, Olmazor koʻchasi, 124-uy</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -11533,7 +11645,7 @@
         </is>
       </c>
       <c r="F174" s="2" t="n">
-        <v>50305390</v>
+        <v>505030539</v>
       </c>
       <c r="G174" s="2" t="n">
         <v>919510536</v>
@@ -11599,10 +11711,10 @@
         </is>
       </c>
       <c r="F175" s="2" t="n">
-        <v>855815350</v>
+        <v>885581535</v>
       </c>
       <c r="G175" s="2" t="n">
-        <v>863315350</v>
+        <v>886331535</v>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
@@ -11611,7 +11723,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>Yashil diyor mfy, Yashil diyor kuchasi, 118.0</t>
+          <t>Yashil diyor 116, Yashil diyor kuchasi, 118 uy</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -11665,19 +11777,19 @@
         </is>
       </c>
       <c r="F176" s="2" t="n">
-        <v>886061500</v>
+        <v>888606150</v>
       </c>
       <c r="G176" s="2" t="n">
-        <v>761500919</v>
+        <v>908776150</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shaxrisabz tumani</t>
         </is>
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>Meraki MFY, NAVOIY KÖCHASI, 48.0</t>
+          <t>Meraki MFY, NAVOIY KÖCHASI, 48-uy</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -11738,7 +11850,7 @@
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz tumani</t>
         </is>
       </c>
       <c r="I177" s="2" t="inlineStr">
@@ -11797,14 +11909,14 @@
         </is>
       </c>
       <c r="F178" s="2" t="n">
-        <v>315225770</v>
+        <v>931522577</v>
       </c>
       <c r="G178" s="2" t="n">
         <v>770867725</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Yakkabog' tumani</t>
+          <t>Qashqadaryo, Yakkaboğ tumani</t>
         </is>
       </c>
       <c r="I178" s="2" t="inlineStr">
@@ -11863,14 +11975,14 @@
         </is>
       </c>
       <c r="F179" s="2" t="n">
-        <v>702090660</v>
+        <v>770209066</v>
       </c>
       <c r="G179" s="2" t="n">
         <v>976175037</v>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I179" s="2" t="inlineStr">
@@ -11975,43 +12087,43 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>Uzoqova Fazilat Nurali qizi</t>
+          <t>Xolmurodova Sabina A'zam qizi</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>40712902560079</t>
+          <t>61604065590015</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>AE4385291</t>
+          <t>AD2922676</t>
         </is>
       </c>
       <c r="F181" s="2" t="n">
-        <v>938918590</v>
+        <v>908810610</v>
       </c>
       <c r="G181" s="2" t="n">
-        <v>976350269</v>
+        <v>908631674</v>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Shahrisabz shahar</t>
         </is>
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>Shamaton MFY, Yangiobod1, 111 uy</t>
+          <t>Fayzabod MFY, Quruvchilar ko'chasi, 73-uy</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
         <is>
-          <t>Qamashi tumani 8-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Shahrisabz tumani 15-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="K181" s="2" t="inlineStr">
         <is>
-          <t>General Secondary School No. 8, Qamashi District</t>
+          <t>General Secondary School No. 15, Shahrisabz District</t>
         </is>
       </c>
       <c r="L181" s="2" t="inlineStr">
@@ -12021,12 +12133,12 @@
       </c>
       <c r="M181" s="2" t="inlineStr">
         <is>
-          <t>O'R-A 5263487</t>
+          <t>UM 02172469</t>
         </is>
       </c>
       <c r="N181" s="2" t="inlineStr">
         <is>
-          <t>1997-2008</t>
+          <t>2013-2024</t>
         </is>
       </c>
     </row>
@@ -12041,43 +12153,43 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>Xolmurodova Sabina A'zam qizi</t>
+          <t>Yahyomurodova Gulsanam Akmal qizi</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>61604065590015</t>
+          <t>62802085680012</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>AD2922676</t>
+          <t>AE4629898</t>
         </is>
       </c>
       <c r="F182" s="2" t="n">
-        <v>908810610</v>
+        <v>773710028</v>
       </c>
       <c r="G182" s="2" t="n">
-        <v>908631674</v>
+        <v>956652882</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Shahrisabz shahri</t>
+          <t>Qashqadaryo, Kitob tumani</t>
         </is>
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>Fayzabod MFY, Quruvchilar ko'chasi, 73-uy</t>
+          <t>Oqsuv MFY, Nimgi qishlog'i, 156uy</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
         <is>
-          <t>Shahrisabz tumani 15-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Kitob tumani 46-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="K182" s="2" t="inlineStr">
         <is>
-          <t>General Secondary School No. 15, Shahrisabz District</t>
+          <t>General Secondary School No. 46, Kitob District</t>
         </is>
       </c>
       <c r="L182" s="2" t="inlineStr">
@@ -12087,12 +12199,12 @@
       </c>
       <c r="M182" s="2" t="inlineStr">
         <is>
-          <t>UM 02172469</t>
+          <t>UM 03729356</t>
         </is>
       </c>
       <c r="N182" s="2" t="inlineStr">
         <is>
-          <t>2013-2024</t>
+          <t>2015-2026</t>
         </is>
       </c>
     </row>
@@ -12107,43 +12219,43 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>Yahyomurodova Gulsanam Akmal qizi</t>
+          <t>Zarifova Marjona Samijon qizi</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>62802085680012</t>
+          <t>63007085680074</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>AE4629898</t>
+          <t>AE4688777</t>
         </is>
       </c>
       <c r="F183" s="2" t="n">
-        <v>737100280</v>
+        <v>875613002</v>
       </c>
       <c r="G183" s="2" t="n">
-        <v>566528820</v>
+        <v>905181884</v>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
-          <t>Qashqadaryo, Kitob tumani</t>
+          <t>Qashqadaryo, Kiuob tumani</t>
         </is>
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>Oqsuv MFY, Yoshlar kuchasi, 156-uy</t>
+          <t>Ulubek MFY, Oʻrikzor koʻchasi, 23-uy</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
         <is>
-          <t>Kitob tumani 46-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Kitob tumani 32-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="K183" s="2" t="inlineStr">
         <is>
-          <t>General Secondary School No. 46, Kitob District</t>
+          <t>General Secondary School No. 32, Kitob District</t>
         </is>
       </c>
       <c r="L183" s="2" t="inlineStr">
@@ -12153,76 +12265,10 @@
       </c>
       <c r="M183" s="2" t="inlineStr">
         <is>
-          <t>UM 03729356</t>
+          <t>UM 03729007</t>
         </is>
       </c>
       <c r="N183" s="2" t="inlineStr">
-        <is>
-          <t>2015-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="184" ht="15.75" customHeight="1">
-      <c r="A184" s="2" t="n">
-        <v>181</v>
-      </c>
-      <c r="B184" s="2" t="inlineStr">
-        <is>
-          <t>26-06</t>
-        </is>
-      </c>
-      <c r="C184" s="2" t="inlineStr">
-        <is>
-          <t>Zarifova Marjona Samijon qizi</t>
-        </is>
-      </c>
-      <c r="D184" s="2" t="inlineStr">
-        <is>
-          <t>63007085680074</t>
-        </is>
-      </c>
-      <c r="E184" s="2" t="inlineStr">
-        <is>
-          <t>AE4688777</t>
-        </is>
-      </c>
-      <c r="F184" s="2" t="n">
-        <v>756130020</v>
-      </c>
-      <c r="G184" s="2" t="n">
-        <v>51818840</v>
-      </c>
-      <c r="H184" s="2" t="inlineStr">
-        <is>
-          <t>Qashqadaryo, Kitob tumani</t>
-        </is>
-      </c>
-      <c r="I184" s="2" t="inlineStr">
-        <is>
-          <t>Ulugʻbek MFY, Urigzor koʻchasi, 23 -uy</t>
-        </is>
-      </c>
-      <c r="J184" s="2" t="inlineStr">
-        <is>
-          <t>Kitob tumani 32-sonli umumiy o'rta ta'lim maktabi</t>
-        </is>
-      </c>
-      <c r="K184" s="2" t="inlineStr">
-        <is>
-          <t>General Secondary School No. 32, Kitob District</t>
-        </is>
-      </c>
-      <c r="L184" s="2" t="inlineStr">
-        <is>
-          <t>Maktab</t>
-        </is>
-      </c>
-      <c r="M184" s="2" t="inlineStr">
-        <is>
-          <t>UM 03729007</t>
-        </is>
-      </c>
-      <c r="N184" s="2" t="inlineStr">
         <is>
           <t>2015-2026</t>
         </is>

</xml_diff>